<commit_message>
Added OLED display firmware
</commit_message>
<xml_diff>
--- a/Firmware/signals.xlsx
+++ b/Firmware/signals.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="169">
   <si>
     <t xml:space="preserve">SIGNAL </t>
   </si>
@@ -517,6 +517,12 @@
   </si>
   <si>
     <t>Byte</t>
+  </si>
+  <si>
+    <t>work led L</t>
+  </si>
+  <si>
+    <t>work led R</t>
   </si>
 </sst>
 </file>
@@ -904,6 +910,9 @@
       <c r="D6">
         <v>0</v>
       </c>
+      <c r="F6" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
@@ -914,6 +923,9 @@
       </c>
       <c r="D7">
         <v>1</v>
+      </c>
+      <c r="F7" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">

</xml_diff>